<commit_message>
update data dictionary with iso_lip_correction and remove sd as this is now collected in data_type
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v19_long.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v19_long.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1954295-D6F7-1144-AAFC-1E0B51918B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E0CBB3-E13B-3541-9A7D-8D44CFF84267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19000" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="tbl_samples" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_dictionary!$A$4:$D$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_dictionary!$A$4:$D$74</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="294">
   <si>
     <t>Field Name</t>
   </si>
@@ -1212,6 +1212,12 @@
   <si>
     <t>Whether the sample is an Individual, Composite, Mean, SD, or Equation</t>
   </si>
+  <si>
+    <t xml:space="preserve">The type of lipid correction done for isotope values </t>
+  </si>
+  <si>
+    <t>as in: bulk; format: character</t>
+  </si>
 </sst>
 </file>
 
@@ -1905,7 +1911,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDB0B4B-8041-E244-B061-95D35DE0CD3B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
@@ -2832,13 +2838,13 @@
         <v>39</v>
       </c>
       <c r="B68" s="30" t="s">
-        <v>36</v>
+        <v>215</v>
       </c>
       <c r="C68" s="30" t="s">
-        <v>62</v>
+        <v>293</v>
       </c>
       <c r="D68" s="30" t="s">
-        <v>57</v>
+        <v>292</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2846,13 +2852,13 @@
         <v>39</v>
       </c>
       <c r="B69" s="30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C69" s="30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D69" s="30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
@@ -2860,13 +2866,13 @@
         <v>39</v>
       </c>
       <c r="B70" s="30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C70" s="30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
@@ -2874,13 +2880,13 @@
         <v>39</v>
       </c>
       <c r="B71" s="30" t="s">
-        <v>218</v>
+        <v>38</v>
       </c>
       <c r="C71" s="30" t="s">
-        <v>222</v>
+        <v>64</v>
       </c>
       <c r="D71" s="30" t="s">
-        <v>219</v>
+        <v>59</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -2888,13 +2894,13 @@
         <v>39</v>
       </c>
       <c r="B72" s="30" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C72" s="30" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D72" s="30" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2902,195 +2908,195 @@
         <v>39</v>
       </c>
       <c r="B73" s="30" t="s">
-        <v>144</v>
+        <v>221</v>
       </c>
       <c r="C73" s="30" t="s">
-        <v>145</v>
+        <v>223</v>
       </c>
       <c r="D73" s="30" t="s">
-        <v>146</v>
+        <v>220</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B74" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="C74" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="D74" s="30" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="30" t="s">
         <v>224</v>
       </c>
-      <c r="B74" s="30" t="s">
+      <c r="B75" s="30" t="s">
         <v>225</v>
       </c>
-      <c r="C74" s="30" t="s">
+      <c r="C75" s="30" t="s">
         <v>226</v>
       </c>
-      <c r="D74" s="30" t="s">
+      <c r="D75" s="30" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A75" s="33" t="s">
-        <v>224</v>
-      </c>
-      <c r="B75" s="33" t="s">
-        <v>228</v>
-      </c>
-      <c r="C75" s="33" t="s">
-        <v>229</v>
-      </c>
-      <c r="D75" s="33" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A76" s="33" t="s">
         <v>224</v>
       </c>
       <c r="B76" s="33" t="s">
+        <v>228</v>
+      </c>
+      <c r="C76" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="D76" s="33" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="B77" s="33" t="s">
         <v>231</v>
       </c>
-      <c r="C76" s="33" t="s">
+      <c r="C77" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="D76" s="33" t="s">
+      <c r="D77" s="33" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A77" s="33" t="s">
-        <v>234</v>
-      </c>
-      <c r="B77" s="34" t="s">
-        <v>235</v>
-      </c>
-      <c r="C77" s="33" t="s">
-        <v>236</v>
-      </c>
-      <c r="D77" s="33" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A78" s="33" t="s">
         <v>234</v>
       </c>
       <c r="B78" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="C78" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="D78" s="33" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+      <c r="A79" s="33" t="s">
+        <v>234</v>
+      </c>
+      <c r="B79" s="34" t="s">
         <v>238</v>
       </c>
-      <c r="C78" s="33" t="s">
+      <c r="C79" s="33" t="s">
         <v>239</v>
       </c>
-      <c r="D78" s="33" t="s">
+      <c r="D79" s="33" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="30" t="s">
-        <v>234</v>
-      </c>
-      <c r="B79" s="35" t="s">
-        <v>241</v>
-      </c>
-      <c r="C79" s="30" t="s">
-        <v>242</v>
-      </c>
-      <c r="D79" s="30" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="30" t="s">
-        <v>244</v>
-      </c>
-      <c r="B80" s="30" t="s">
-        <v>245</v>
+        <v>234</v>
+      </c>
+      <c r="B80" s="35" t="s">
+        <v>241</v>
       </c>
       <c r="C80" s="30" t="s">
-        <v>287</v>
-      </c>
-      <c r="D80" s="33" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+        <v>242</v>
+      </c>
+      <c r="D80" s="30" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="30" t="s">
         <v>244</v>
       </c>
       <c r="B81" s="30" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C81" s="30" t="s">
-        <v>239</v>
+        <v>287</v>
       </c>
       <c r="D81" s="33" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A82" s="30" t="s">
         <v>244</v>
       </c>
       <c r="B82" s="30" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C82" s="30" t="s">
-        <v>283</v>
+        <v>239</v>
       </c>
       <c r="D82" s="33" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="30" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="B83" s="30" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C83" s="30" t="s">
-        <v>279</v>
-      </c>
-      <c r="D83" s="30" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+        <v>283</v>
+      </c>
+      <c r="D83" s="33" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="30" t="s">
         <v>266</v>
       </c>
-      <c r="B84" s="40" t="s">
-        <v>276</v>
+      <c r="B84" s="30" t="s">
+        <v>251</v>
       </c>
       <c r="C84" s="30" t="s">
-        <v>280</v>
-      </c>
-      <c r="D84" s="33" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+        <v>279</v>
+      </c>
+      <c r="D84" s="30" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A85" s="30" t="s">
         <v>266</v>
       </c>
       <c r="B85" s="40" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C85" s="30" t="s">
-        <v>281</v>
-      </c>
-      <c r="D85" s="30" t="s">
-        <v>282</v>
+        <v>280</v>
+      </c>
+      <c r="D85" s="33" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="B86" s="30" t="s">
-        <v>253</v>
+        <v>266</v>
+      </c>
+      <c r="B86" s="40" t="s">
+        <v>277</v>
       </c>
       <c r="C86" s="30" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D86" s="30" t="s">
-        <v>254</v>
+        <v>282</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -3098,13 +3104,13 @@
         <v>264</v>
       </c>
       <c r="B87" s="30" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C87" s="30" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -3112,13 +3118,13 @@
         <v>264</v>
       </c>
       <c r="B88" s="30" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C88" s="30" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="D88" s="30" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
@@ -3126,13 +3132,13 @@
         <v>264</v>
       </c>
       <c r="B89" s="30" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="C89" s="30" t="s">
-        <v>286</v>
+        <v>257</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
@@ -3140,12 +3146,26 @@
         <v>264</v>
       </c>
       <c r="B90" s="30" t="s">
+        <v>259</v>
+      </c>
+      <c r="C90" s="30" t="s">
+        <v>286</v>
+      </c>
+      <c r="D90" s="30" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="30" t="s">
+        <v>264</v>
+      </c>
+      <c r="B91" s="30" t="s">
         <v>261</v>
       </c>
-      <c r="C90" s="30" t="s">
+      <c r="C91" s="30" t="s">
         <v>262</v>
       </c>
-      <c r="D90" s="30" t="s">
+      <c r="D91" s="30" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>